<commit_message>
chore: m066 stats 갱신 + filled Excel 업데이트
- pfm26-m066-stats.json: rebuild-atomic 후 최신 통계 반영
  (L1F 21→28, FC 98→111, FL 163→338, FE 24→41)
- filled Excel: 바이너리 업데이트

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master-fmea/master_import_12inch_AuBump_filled.xlsx
+++ b/data/master-fmea/master_import_12inch_AuBump_filled.xlsx
@@ -38,7 +38,29 @@
     <t>Au Bump 제품특성(높이·순도·외관)이 자사 공정 수율 기준을 충족하는 Wafer를 제공한다</t>
   </si>
   <si>
-    <t>Au Bump 높이 규격(Bump Height Spec, μm)</t>
+    <r>
+      <t xml:space="preserve">Au Bump 높이 규격 (Bump Height Spec, </t>
+    </r>
+    <r>
+      <rPr>
+        <charset val="161"/>
+        <color theme="1"/>
+        <family val="2"/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>μ</t>
+    </r>
+    <r>
+      <rPr>
+        <color theme="1"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+      </rPr>
+      <t>m)</t>
+    </r>
   </si>
   <si>
     <t>Particle 오염으로 인한 제품 특성 이상</t>
@@ -107,7 +129,29 @@
     <t>고객 납품 기준(높이·외관·포장)을 충족하는 Wafer를 제공한다</t>
   </si>
   <si>
-    <t>Au Bump 높이 고객 출하 규격(Customer Bump Height Spec, μm)</t>
+    <r>
+      <t xml:space="preserve">Au Bump 높이 고객 출하 규격 (Customer Bump Height Spec, </t>
+    </r>
+    <r>
+      <rPr>
+        <charset val="161"/>
+        <color theme="1"/>
+        <family val="2"/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>μ</t>
+    </r>
+    <r>
+      <rPr>
+        <color theme="1"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+        <sz val="11"/>
+        <rFont val="맑은 고딕"/>
+      </rPr>
+      <t>m)</t>
+    </r>
   </si>
   <si>
     <t>IMC 과성장에 의한 접합부 열화</t>

</xml_diff>